<commit_message>
dividindo workflows e inserindo logs
</commit_message>
<xml_diff>
--- a/dados/ACME_Dados.xlsx
+++ b/dados/ACME_Dados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://suzano-my.sharepoint.com/personal/julianobs_suzano_com_br/Documents/Area Dev/GitHub/UiPath/ExtracaoDadosWeb/dados/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="13" documentId="11_D8261291F1A51D60D742301D8CFE11A0A62C7127" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{37FEA429-D11E-4A37-9183-DCD8F960F4D6}"/>
+  <xr:revisionPtr revIDLastSave="15" documentId="11_D8261291F1A51D60D742301D8CFE11A0A62C7127" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0E1C5F81-8C87-4984-8810-F5A887CEBD18}"/>
   <x:bookViews>
     <x:workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="0" activeTab="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </x:bookViews>
@@ -197,6 +197,156 @@
   </x:si>
   <x:si>
     <x:t>2017-08-01</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://acme-test.uipath.com/work-items/108326246</x:t>
+  </x:si>
+  <x:si>
+    <x:t>108326246</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2021-04-26</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://acme-test.uipath.com/work-items/108326216</x:t>
+  </x:si>
+  <x:si>
+    <x:t>108326216</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2018-09-13</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://acme-test.uipath.com/work-items/108326227</x:t>
+  </x:si>
+  <x:si>
+    <x:t>108326227</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2018-12-26</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://acme-test.uipath.com/work-items/108326231</x:t>
+  </x:si>
+  <x:si>
+    <x:t>108326231</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2020-11-15</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://acme-test.uipath.com/work-items/108326241</x:t>
+  </x:si>
+  <x:si>
+    <x:t>108326241</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2018-12-09</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://acme-test.uipath.com/work-items/108326247</x:t>
+  </x:si>
+  <x:si>
+    <x:t>108326247</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2021-11-14</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://acme-test.uipath.com/work-items/108326236</x:t>
+  </x:si>
+  <x:si>
+    <x:t>108326236</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2025-05-11</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://acme-test.uipath.com/work-items/108326233</x:t>
+  </x:si>
+  <x:si>
+    <x:t>108326233</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2018-04-06</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://acme-test.uipath.com/work-items/108326217</x:t>
+  </x:si>
+  <x:si>
+    <x:t>108326217</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2017-10-01</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://acme-test.uipath.com/work-items/108326239</x:t>
+  </x:si>
+  <x:si>
+    <x:t>108326239</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2019-05-08</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://acme-test.uipath.com/work-items/108326229</x:t>
+  </x:si>
+  <x:si>
+    <x:t>108326229</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2018-06-27</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://acme-test.uipath.com/work-items/108326238</x:t>
+  </x:si>
+  <x:si>
+    <x:t>108326238</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://acme-test.uipath.com/work-items/108326245</x:t>
+  </x:si>
+  <x:si>
+    <x:t>108326245</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2025-05-01</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://acme-test.uipath.com/work-items/108326242</x:t>
+  </x:si>
+  <x:si>
+    <x:t>108326242</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2019-02-12</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://acme-test.uipath.com/work-items/108326226</x:t>
+  </x:si>
+  <x:si>
+    <x:t>108326226</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2019-01-08</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://acme-test.uipath.com/work-items/108326223</x:t>
+  </x:si>
+  <x:si>
+    <x:t>108326223</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2017-03-06</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://acme-test.uipath.com/work-items/108326234</x:t>
+  </x:si>
+  <x:si>
+    <x:t>108326234</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2017-02-21</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -877,6 +1027,346 @@
         <x:v>56</x:v>
       </x:c>
     </x:row>
+    <x:row r="18" spans="1:6">
+      <x:c r="A18" s="0" t="s">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="B18" s="0" t="s">
+        <x:v>58</x:v>
+      </x:c>
+      <x:c r="C18" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D18" s="0" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E18" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F18" s="0" t="s">
+        <x:v>59</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" spans="1:6">
+      <x:c r="A19" s="0" t="s">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="B19" s="0" t="s">
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="C19" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D19" s="0" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E19" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F19" s="0" t="s">
+        <x:v>62</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" spans="1:6">
+      <x:c r="A20" s="0" t="s">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="B20" s="0" t="s">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="C20" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D20" s="0" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E20" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F20" s="0" t="s">
+        <x:v>65</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" spans="1:6">
+      <x:c r="A21" s="0" t="s">
+        <x:v>66</x:v>
+      </x:c>
+      <x:c r="B21" s="0" t="s">
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="C21" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D21" s="0" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E21" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F21" s="0" t="s">
+        <x:v>68</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" spans="1:6">
+      <x:c r="A22" s="0" t="s">
+        <x:v>69</x:v>
+      </x:c>
+      <x:c r="B22" s="0" t="s">
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="C22" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D22" s="0" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E22" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F22" s="0" t="s">
+        <x:v>71</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" spans="1:6">
+      <x:c r="A23" s="0" t="s">
+        <x:v>72</x:v>
+      </x:c>
+      <x:c r="B23" s="0" t="s">
+        <x:v>73</x:v>
+      </x:c>
+      <x:c r="C23" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D23" s="0" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E23" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F23" s="0" t="s">
+        <x:v>74</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" spans="1:6">
+      <x:c r="A24" s="0" t="s">
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="B24" s="0" t="s">
+        <x:v>76</x:v>
+      </x:c>
+      <x:c r="C24" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D24" s="0" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E24" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F24" s="0" t="s">
+        <x:v>77</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" spans="1:6">
+      <x:c r="A25" s="0" t="s">
+        <x:v>78</x:v>
+      </x:c>
+      <x:c r="B25" s="0" t="s">
+        <x:v>79</x:v>
+      </x:c>
+      <x:c r="C25" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D25" s="0" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E25" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F25" s="0" t="s">
+        <x:v>80</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" spans="1:6">
+      <x:c r="A26" s="0" t="s">
+        <x:v>81</x:v>
+      </x:c>
+      <x:c r="B26" s="0" t="s">
+        <x:v>82</x:v>
+      </x:c>
+      <x:c r="C26" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D26" s="0" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E26" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F26" s="0" t="s">
+        <x:v>83</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" spans="1:6">
+      <x:c r="A27" s="0" t="s">
+        <x:v>84</x:v>
+      </x:c>
+      <x:c r="B27" s="0" t="s">
+        <x:v>85</x:v>
+      </x:c>
+      <x:c r="C27" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D27" s="0" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E27" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F27" s="0" t="s">
+        <x:v>86</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" spans="1:6">
+      <x:c r="A28" s="0" t="s">
+        <x:v>87</x:v>
+      </x:c>
+      <x:c r="B28" s="0" t="s">
+        <x:v>88</x:v>
+      </x:c>
+      <x:c r="C28" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D28" s="0" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E28" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F28" s="0" t="s">
+        <x:v>89</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" spans="1:6">
+      <x:c r="A29" s="0" t="s">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="B29" s="0" t="s">
+        <x:v>91</x:v>
+      </x:c>
+      <x:c r="C29" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D29" s="0" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E29" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F29" s="0" t="s">
+        <x:v>47</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" spans="1:6">
+      <x:c r="A30" s="0" t="s">
+        <x:v>92</x:v>
+      </x:c>
+      <x:c r="B30" s="0" t="s">
+        <x:v>93</x:v>
+      </x:c>
+      <x:c r="C30" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D30" s="0" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E30" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F30" s="0" t="s">
+        <x:v>94</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" spans="1:6">
+      <x:c r="A31" s="0" t="s">
+        <x:v>95</x:v>
+      </x:c>
+      <x:c r="B31" s="0" t="s">
+        <x:v>96</x:v>
+      </x:c>
+      <x:c r="C31" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D31" s="0" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E31" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F31" s="0" t="s">
+        <x:v>97</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" spans="1:6">
+      <x:c r="A32" s="0" t="s">
+        <x:v>98</x:v>
+      </x:c>
+      <x:c r="B32" s="0" t="s">
+        <x:v>99</x:v>
+      </x:c>
+      <x:c r="C32" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D32" s="0" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E32" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F32" s="0" t="s">
+        <x:v>100</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" spans="1:6">
+      <x:c r="A33" s="0" t="s">
+        <x:v>101</x:v>
+      </x:c>
+      <x:c r="B33" s="0" t="s">
+        <x:v>102</x:v>
+      </x:c>
+      <x:c r="C33" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D33" s="0" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E33" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F33" s="0" t="s">
+        <x:v>103</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" spans="1:6">
+      <x:c r="A34" s="0" t="s">
+        <x:v>104</x:v>
+      </x:c>
+      <x:c r="B34" s="0" t="s">
+        <x:v>105</x:v>
+      </x:c>
+      <x:c r="C34" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D34" s="0" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E34" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F34" s="0" t="s">
+        <x:v>106</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>